<commit_message>
OUT_last_timestep_VP to handle tile number tag
</commit_message>
<xml_diff>
--- a/CryoGrid/CryoGridCommunity_results/TEST/accelerated_spinup/TILES_ACCELERATED.xlsx
+++ b/CryoGrid/CryoGridCommunity_results/TEST/accelerated_spinup/TILES_ACCELERATED.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Utilisateurs\pozsgayv\Documents\CryoGrid_VP_Workflow\CryoGrid\CryoGridCommunity_results\templates\accelerated_spinup\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Utilisateurs\pozsgayv\Documents\CryoGrid_VP_Workflow\CryoGrid\CryoGridCommunity_results\TEST\accelerated_spinup\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C94ECA68-1136-47F0-8B5A-1E05DC2E2950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38CE66C8-A340-420F-BCB6-2F500D304771}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3300" yWindow="3110" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -737,91 +737,91 @@
     <t>include_Xice</t>
   </si>
   <si>
+    <t>horizon_angles</t>
+  </si>
+  <si>
+    <t>snow_property_function</t>
+  </si>
+  <si>
+    <t>for hydrology</t>
+  </si>
+  <si>
+    <t>only for soil; e-folding depth of transpiration reduction with depth [m]</t>
+  </si>
+  <si>
+    <t>only for soil; e-folding constant of evaporation reduction reduction with depth [m]</t>
+  </si>
+  <si>
+    <t>if empty, compute automatically as function of mean pressure, i.e. 0.2./60 day^-1 for altitude 870hPa</t>
+  </si>
+  <si>
+    <t>lateral framework always needed at elast LATERAL_1D</t>
+  </si>
+  <si>
+    <t>satHydraulicConductivity</t>
+  </si>
+  <si>
+    <t>field_capacity should be inferior than waterice</t>
+  </si>
+  <si>
+    <t>OUT_regridded</t>
+  </si>
+  <si>
+    <t>relative2surface</t>
+  </si>
+  <si>
+    <t>if 0, in m a.s.l; if 1, elevation relative to surface with upper and lower POSITIVE</t>
+  </si>
+  <si>
+    <t>upper elevation of output domain, in m a.s.l if relative2surface=0, else in (positive) meters above the surface if =1; must match altitude in TILE!</t>
+  </si>
+  <si>
+    <t>lower elevation of output domain, in m a.s.l if relative2surface=0, else in (positive) meters below the surface if =1; must match altitude in TILE!</t>
+  </si>
+  <si>
+    <t>same as OUT_TwaterIce, but you can set elevations relative to the surface elevation, which is much more user-friendly</t>
+  </si>
+  <si>
+    <t>OUT_all_lateral</t>
+  </si>
+  <si>
+    <t>TILE_1D</t>
+  </si>
+  <si>
+    <t>not necessary unless user wants an output, but could be OUT_do_nothing instead</t>
+  </si>
+  <si>
+    <t>restart_OUT_last_timestep</t>
+  </si>
+  <si>
+    <t>restart_file_path</t>
+  </si>
+  <si>
+    <t>restart_file_name</t>
+  </si>
+  <si>
+    <t>adapt_run_name</t>
+  </si>
+  <si>
+    <t>new_end_time</t>
+  </si>
+  <si>
+    <t>save_timestep</t>
+  </si>
+  <si>
+    <t>timestep that model progress is displayed [days], if empty save final state at the end of the run, so that it can serve as initial condition for new runs</t>
+  </si>
+  <si>
+    <t>use_save_date</t>
+  </si>
+  <si>
+    <t>if 0/false (default), normal behaviour with file being overwritten every save_timestep [days]; if 1/true, then a new file with tile index and spinup index is created to prevent overwriting (uses save_date and save_interval below)</t>
+  </si>
+  <si>
+    <t>OUT_last_timestep_VP</t>
+  </si>
+  <si>
     <t>RUN_1D_POINT_SPINUP</t>
-  </si>
-  <si>
-    <t>horizon_angles</t>
-  </si>
-  <si>
-    <t>snow_property_function</t>
-  </si>
-  <si>
-    <t>for hydrology</t>
-  </si>
-  <si>
-    <t>only for soil; e-folding depth of transpiration reduction with depth [m]</t>
-  </si>
-  <si>
-    <t>only for soil; e-folding constant of evaporation reduction reduction with depth [m]</t>
-  </si>
-  <si>
-    <t>if empty, compute automatically as function of mean pressure, i.e. 0.2./60 day^-1 for altitude 870hPa</t>
-  </si>
-  <si>
-    <t>lateral framework always needed at elast LATERAL_1D</t>
-  </si>
-  <si>
-    <t>satHydraulicConductivity</t>
-  </si>
-  <si>
-    <t>field_capacity should be inferior than waterice</t>
-  </si>
-  <si>
-    <t>OUT_regridded</t>
-  </si>
-  <si>
-    <t>relative2surface</t>
-  </si>
-  <si>
-    <t>if 0, in m a.s.l; if 1, elevation relative to surface with upper and lower POSITIVE</t>
-  </si>
-  <si>
-    <t>upper elevation of output domain, in m a.s.l if relative2surface=0, else in (positive) meters above the surface if =1; must match altitude in TILE!</t>
-  </si>
-  <si>
-    <t>lower elevation of output domain, in m a.s.l if relative2surface=0, else in (positive) meters below the surface if =1; must match altitude in TILE!</t>
-  </si>
-  <si>
-    <t>same as OUT_TwaterIce, but you can set elevations relative to the surface elevation, which is much more user-friendly</t>
-  </si>
-  <si>
-    <t>OUT_all_lateral</t>
-  </si>
-  <si>
-    <t>TILE_1D</t>
-  </si>
-  <si>
-    <t>not necessary unless user wants an output, but could be OUT_do_nothing instead</t>
-  </si>
-  <si>
-    <t>restart_OUT_last_timestep</t>
-  </si>
-  <si>
-    <t>restart_file_path</t>
-  </si>
-  <si>
-    <t>restart_file_name</t>
-  </si>
-  <si>
-    <t>adapt_run_name</t>
-  </si>
-  <si>
-    <t>new_end_time</t>
-  </si>
-  <si>
-    <t>OUT_last_timestep</t>
-  </si>
-  <si>
-    <t>save_timestep</t>
-  </si>
-  <si>
-    <t>timestep that model progress is displayed [days], if empty save final state at the end of the run, so that it can serve as initial condition for new runs</t>
-  </si>
-  <si>
-    <t>use_save_date</t>
-  </si>
-  <si>
-    <t>if 0/false (default), normal behaviour with file being overwritten every save_timestep [days]; if 1/true, then a new file with tile index and spinup index is created to prevent overwriting (uses save_date and save_interval below)</t>
   </si>
 </sst>
 </file>
@@ -1228,7 +1228,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
-        <v>233</v>
+        <v>261</v>
       </c>
       <c r="B3" s="8">
         <v>1</v>
@@ -1258,22 +1258,22 @@
         <v>4</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I6" s="8" t="s">
         <v>5</v>
@@ -1422,7 +1422,7 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="9" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B22" s="9"/>
       <c r="C22" s="5"/>
@@ -1456,7 +1456,7 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="8" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B28" s="8">
         <v>1</v>
@@ -1521,13 +1521,13 @@
         <v>4</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="D36" s="8" t="s">
         <v>5</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
@@ -1705,7 +1705,7 @@
     </row>
     <row r="55" spans="1:4" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B55">
         <v>2</v>
@@ -1717,17 +1717,17 @@
         <v>11</v>
       </c>
       <c r="B57" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="58" spans="1:4" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="59" spans="1:4" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="60" spans="1:4" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.35">
@@ -1760,12 +1760,12 @@
     </row>
     <row r="62" spans="1:4" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="63" spans="1:4" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C63" s="14"/>
       <c r="D63" s="14"/>
@@ -1794,7 +1794,7 @@
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B69" s="9">
         <v>3</v>
@@ -1839,7 +1839,7 @@
         <v>77</v>
       </c>
       <c r="D74" s="8" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="E74" s="8" t="s">
         <v>5</v>
@@ -1891,7 +1891,7 @@
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="8" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B81" s="8">
         <v>4</v>
@@ -1956,7 +1956,7 @@
         <v>4</v>
       </c>
       <c r="C89" s="8" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="D89" s="8" t="s">
         <v>5</v>
@@ -2134,7 +2134,7 @@
     </row>
     <row r="108" spans="1:6" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B108">
         <v>5</v>
@@ -2146,17 +2146,17 @@
         <v>11</v>
       </c>
       <c r="B110" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="111" spans="1:6" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="112" spans="1:6" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="113" spans="1:7" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.35">
@@ -2189,12 +2189,12 @@
     </row>
     <row r="115" spans="1:7" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="116" spans="1:7" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C116" s="14"/>
       <c r="D116" s="14"/>
@@ -2226,7 +2226,7 @@
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A122" s="9" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B122" s="9">
         <v>6</v>
@@ -2294,16 +2294,16 @@
         <v>4</v>
       </c>
       <c r="C128" s="9" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D128" s="9" t="s">
         <v>218</v>
       </c>
       <c r="E128" s="8" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F128" s="8" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="G128" s="9" t="s">
         <v>5</v>
@@ -3072,7 +3072,7 @@
     </row>
     <row r="229" spans="1:4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A229" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="B229">
         <v>1</v>
@@ -3081,10 +3081,10 @@
     <row r="230" spans="1:4" customFormat="1" x14ac:dyDescent="0.35"/>
     <row r="231" spans="1:4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A231" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D231" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="232" spans="1:4" customFormat="1" x14ac:dyDescent="0.35">
@@ -3094,13 +3094,13 @@
     </row>
     <row r="233" spans="1:4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A233" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B233">
         <v>1</v>
       </c>
       <c r="D233" s="2" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="234" spans="1:4" customFormat="1" x14ac:dyDescent="0.35">
@@ -3153,7 +3153,7 @@
     </row>
     <row r="241" spans="1:8" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A241" s="9" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B241" s="9">
         <v>1</v>
@@ -3236,13 +3236,13 @@
     </row>
     <row r="252" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A252" s="8" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B252" s="8">
         <v>1</v>
       </c>
       <c r="D252" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="253" spans="1:8" x14ac:dyDescent="0.35">
@@ -3273,13 +3273,13 @@
     </row>
     <row r="254" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A254" s="8" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B254" s="8">
         <v>0</v>
       </c>
       <c r="D254" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="H254" s="2"/>
     </row>
@@ -3291,7 +3291,7 @@
         <v>24</v>
       </c>
       <c r="D255" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="256" spans="1:8" x14ac:dyDescent="0.35">
@@ -3302,7 +3302,7 @@
         <v>0</v>
       </c>
       <c r="D256" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="257" spans="1:8" x14ac:dyDescent="0.35">
@@ -3643,7 +3643,7 @@
         <v>1</v>
       </c>
       <c r="F299" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="300" spans="1:6" x14ac:dyDescent="0.35">
@@ -3744,13 +3744,13 @@
         <v>118</v>
       </c>
       <c r="H312" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="I312" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="J312" s="2" t="s">
         <v>241</v>
-      </c>
-      <c r="I312" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="J312" s="2" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="313" spans="1:10" x14ac:dyDescent="0.35">
@@ -3913,7 +3913,7 @@
         <v>0.1</v>
       </c>
       <c r="D327" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="328" spans="1:4" x14ac:dyDescent="0.35">
@@ -3927,7 +3927,7 @@
         <v>0.1</v>
       </c>
       <c r="D328" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="329" spans="1:4" x14ac:dyDescent="0.35">
@@ -4623,7 +4623,7 @@
         <v>1E-3</v>
       </c>
       <c r="D393" s="2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="394" spans="1:4" x14ac:dyDescent="0.35">
@@ -4670,7 +4670,7 @@
     </row>
     <row r="397" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A397" s="8" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D397" s="2"/>
     </row>
@@ -4700,7 +4700,7 @@
         <v>1</v>
       </c>
       <c r="D403" s="2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="404" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>